<commit_message>
Update FIRIS forecast 2026-09-04
</commit_message>
<xml_diff>
--- a/data/report/firis_report.xlsx
+++ b/data/report/firis_report.xlsx
@@ -45,13 +45,13 @@
     <font>
       <name val="B Nazanin"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="00000000"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="B Nazanin"/>
       <b val="1"/>
-      <color rgb="00000000"/>
+      <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -64,7 +64,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FB8C00"/>
+        <fgColor rgb="00FDD835"/>
       </patternFill>
     </fill>
     <fill>
@@ -74,7 +74,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FDD835"/>
+        <fgColor rgb="00FB8C00"/>
       </patternFill>
     </fill>
     <fill>
@@ -127,13 +127,13 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -533,7 +533,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
     </row>
@@ -545,7 +545,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>fli_fars_2026-09-03.tif</t>
+          <t>fli_fars_2026-09-04.tif</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>70.2</v>
+        <v>63.76</v>
       </c>
     </row>
     <row r="9">
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>41.61</v>
+        <v>37.63</v>
       </c>
     </row>
     <row r="10">
@@ -609,7 +609,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>زیاد</t>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -718,13 +718,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>48.22</v>
+        <v>42.11</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>35.98</v>
+        <v>26.66</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>63.53</v>
+        <v>60.44</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>24441</v>
@@ -750,13 +750,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>45.9</v>
+        <v>43.82</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>31.59</v>
+        <v>30.26</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>60.77</v>
+        <v>57.48</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>5703</v>
@@ -782,13 +782,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>37.85</v>
+        <v>31.5</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0.43</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>56.89</v>
+        <v>50.76</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>751</v>
@@ -814,13 +814,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>44.15</v>
+        <v>44.49</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>37.15</v>
+        <v>36.83</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>57.63</v>
+        <v>58.44</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>10563</v>
@@ -846,20 +846,20 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>44.39</v>
+        <v>39.63</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>37.41</v>
+        <v>31.35</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>52.81</v>
+        <v>48.87</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>1663</v>
       </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -878,13 +878,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>56.14</v>
+        <v>42.57</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>47.74</v>
+        <v>31.71</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>68.58</v>
+        <v>55.07</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>2137</v>
@@ -910,13 +910,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>33.85</v>
+        <v>36.96</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>1.01</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>55.67</v>
+        <v>55.82</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>1950</v>
@@ -942,20 +942,20 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>45.42</v>
+        <v>36.37</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>35.27</v>
+        <v>29.28</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>58.07</v>
+        <v>50.1</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>187</v>
       </c>
-      <c r="H9" s="4" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -974,20 +974,20 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>43.38</v>
+        <v>37.91</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>33.04</v>
+        <v>30.47</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>55.43</v>
+        <v>50.28</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>1059</v>
       </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -1006,13 +1006,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>43.3</v>
+        <v>41.59</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>33.05</v>
+        <v>28.62</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>61.29</v>
+        <v>58.86</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>3976</v>
@@ -1038,13 +1038,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>44.37</v>
+        <v>42.77</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>34.59</v>
+        <v>28.46</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>59.17</v>
+        <v>58.81</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>5465</v>
@@ -1070,20 +1070,20 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>41.76</v>
+        <v>38.61</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>28.55</v>
+        <v>27.65</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>55.85</v>
+        <v>53.19</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>6849</v>
       </c>
-      <c r="H13" s="4" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -1102,13 +1102,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>22.71</v>
+        <v>22.17</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>1.06</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>31.86</v>
+        <v>32.82</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>79</v>
@@ -1134,13 +1134,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>26.99</v>
+        <v>27.11</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>0.45</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>47.41</v>
+        <v>49.01</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>932</v>
@@ -1166,13 +1166,13 @@
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>46.98</v>
+        <v>42.71</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>37.33</v>
+        <v>30.04</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>64.63</v>
+        <v>57.58</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>4808</v>
@@ -1198,13 +1198,13 @@
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>27.12</v>
+        <v>27.18</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>1.32</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>49.6</v>
+        <v>48.27</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>4944</v>
@@ -1230,20 +1230,20 @@
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>46.14</v>
+        <v>33.94</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>0.65</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>62.8</v>
+        <v>53.49</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>5180</v>
       </c>
-      <c r="H18" s="4" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -1262,13 +1262,13 @@
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>32.32</v>
+        <v>32.52</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>0.59</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>45.26</v>
+        <v>47.03</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>3925</v>
@@ -1294,13 +1294,13 @@
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>55.55</v>
+        <v>40.55</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>45.86</v>
+        <v>29.84</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>67.69</v>
+        <v>51.32</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>657</v>
@@ -1326,13 +1326,13 @@
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>47.37</v>
+        <v>43.48</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>35.37</v>
+        <v>32.16</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>61.3</v>
+        <v>58.11</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>6257</v>
@@ -1358,13 +1358,13 @@
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>19.08</v>
+        <v>18.37</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>3.47</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>44.62</v>
+        <v>42.08</v>
       </c>
       <c r="G22" s="1" t="n">
         <v>70</v>
@@ -1458,13 +1458,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>47.31</v>
+        <v>42.25</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>39.03</v>
+        <v>33.23</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>59.94</v>
+        <v>54.88</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>2293</v>
@@ -1490,13 +1490,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>47.3</v>
+        <v>42.45</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>38.68</v>
+        <v>33.04</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>64.01000000000001</v>
+        <v>62</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>4823</v>
@@ -1522,13 +1522,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>23.08</v>
+        <v>23.52</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0.55</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>42.68</v>
+        <v>44.07</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>868</v>
@@ -1554,13 +1554,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>44.25</v>
+        <v>40.22</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>36.53</v>
+        <v>32.44</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>55.74</v>
+        <v>51.77</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>466</v>
@@ -1586,13 +1586,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>30.38</v>
+        <v>24.98</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>57.94</v>
+        <v>47.01</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>2048</v>
@@ -1618,13 +1618,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>38.59</v>
+        <v>35.18</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>6.54</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>46.91</v>
+        <v>43.22</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>173</v>
@@ -1650,20 +1650,20 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>41.02</v>
+        <v>39.51</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>30.35</v>
+        <v>28.44</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>58.67</v>
+        <v>56.32</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>7042</v>
       </c>
-      <c r="H8" s="4" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -1682,13 +1682,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>28.41</v>
+        <v>25.58</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>9.050000000000001</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>56.89</v>
+        <v>50.76</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>66</v>
@@ -1714,13 +1714,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>42.9</v>
+        <v>41.55</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>32.88</v>
+        <v>32.24</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>57.97</v>
+        <v>55.29</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>6931</v>
@@ -1746,13 +1746,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>49.41</v>
+        <v>44.29</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>40.57</v>
+        <v>28.43</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>62.87</v>
+        <v>57.55</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>5654</v>
@@ -1778,20 +1778,20 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>46.86</v>
+        <v>38.39</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>3.99</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>70.2</v>
+        <v>55.18</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>16529</v>
       </c>
-      <c r="H12" s="4" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -1810,20 +1810,20 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>46.72</v>
+        <v>37.18</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>4.03</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>62.22</v>
+        <v>54.15</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>5265</v>
       </c>
-      <c r="H13" s="4" t="inlineStr">
-        <is>
-          <t>زیاد</t>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -1842,13 +1842,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>46.51</v>
+        <v>43.8</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>36.75</v>
+        <v>33.88</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>60.14</v>
+        <v>57.25</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>2311</v>
@@ -1874,13 +1874,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>49.72</v>
+        <v>46.8</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>42.12</v>
+        <v>38.52</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>62.43</v>
+        <v>59.96</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>1185</v>
@@ -1954,10 +1954,10 @@
         <v>20</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>39403</v>
+        <v>40236</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>4.36</v>
+        <v>4.45</v>
       </c>
     </row>
     <row r="3">
@@ -1973,10 +1973,10 @@
         <v>40</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>246062</v>
+        <v>476074</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>27.2</v>
+        <v>52.62</v>
       </c>
     </row>
     <row r="4">
@@ -1992,10 +1992,10 @@
         <v>60</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>616574</v>
+        <v>388373</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>68.15000000000001</v>
+        <v>42.93</v>
       </c>
     </row>
     <row r="5">
@@ -2011,10 +2011,10 @@
         <v>80</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>2714</v>
+        <v>70</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>0.3</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Update FIRIS forecast 2026-09-05
</commit_message>
<xml_diff>
--- a/data/report/firis_report.xlsx
+++ b/data/report/firis_report.xlsx
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>63.59</v>
+        <v>65.95</v>
       </c>
     </row>
     <row r="9">
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>37.07</v>
+        <v>37.03</v>
       </c>
     </row>
     <row r="10">
@@ -718,13 +718,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>40.6</v>
+        <v>40.59</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>28.09</v>
+        <v>30.07</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>56.67</v>
+        <v>56.46</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>24441</v>
@@ -750,13 +750,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>42.82</v>
+        <v>40.8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>28.5</v>
+        <v>27.05</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>57.03</v>
+        <v>55.04</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>5703</v>
@@ -782,13 +782,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>26.03</v>
+        <v>25</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0.43</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>42.89</v>
+        <v>41.93</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>751</v>
@@ -814,13 +814,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>41.99</v>
+        <v>43.21</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>33.83</v>
+        <v>35.15</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>55.83</v>
+        <v>56.46</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>10563</v>
@@ -846,13 +846,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>38.91</v>
+        <v>36.91</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>33</v>
+        <v>31.01</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>48.25</v>
+        <v>45.76</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>1663</v>
@@ -878,13 +878,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>47.48</v>
+        <v>47.78</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>38.66</v>
+        <v>39.21</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>58.29</v>
+        <v>59.2</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>2137</v>
@@ -910,13 +910,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>35.93</v>
+        <v>36.32</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>1.01</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>53.95</v>
+        <v>54.68</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>1950</v>
@@ -942,13 +942,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>34.52</v>
+        <v>32.72</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>28.08</v>
+        <v>26.42</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>47.26</v>
+        <v>44.43</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>187</v>
@@ -974,13 +974,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>33.93</v>
+        <v>31.17</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>26.4</v>
+        <v>25.61</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>45.42</v>
+        <v>41.3</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>1059</v>
@@ -1006,13 +1006,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>39.36</v>
+        <v>39.89</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>28.45</v>
+        <v>27.59</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>54.72</v>
+        <v>56.21</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>3976</v>
@@ -1038,13 +1038,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>44.33</v>
+        <v>42.82</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>33.64</v>
+        <v>32.55</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>59.89</v>
+        <v>58.25</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>5465</v>
@@ -1070,13 +1070,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>42.12</v>
+        <v>42.26</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>29.55</v>
+        <v>28.49</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>59.39</v>
+        <v>60.92</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>6849</v>
@@ -1102,13 +1102,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>24.14</v>
+        <v>24.44</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>1.06</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>35.74</v>
+        <v>35.71</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>79</v>
@@ -1134,13 +1134,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>27.87</v>
+        <v>29.38</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>0.45</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>46.59</v>
+        <v>49.18</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>932</v>
@@ -1166,13 +1166,13 @@
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>41.68</v>
+        <v>40.76</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>29.62</v>
+        <v>31.15</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>56.66</v>
+        <v>55.92</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>4808</v>
@@ -1198,13 +1198,13 @@
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>26.19</v>
+        <v>27.09</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>1.32</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>47.13</v>
+        <v>48.7</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>4944</v>
@@ -1230,13 +1230,13 @@
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>34.19</v>
+        <v>33.13</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>0.65</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>52</v>
+        <v>48.85</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>5180</v>
@@ -1262,13 +1262,13 @@
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>34.33</v>
+        <v>32.33</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>0.59</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>49.26</v>
+        <v>46.73</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>3925</v>
@@ -1294,13 +1294,13 @@
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>45.28</v>
+        <v>43.55</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>35.68</v>
+        <v>33.16</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>55.68</v>
+        <v>55.25</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>657</v>
@@ -1326,13 +1326,13 @@
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>42.14</v>
+        <v>42.24</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>30.97</v>
+        <v>30.92</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>56.66</v>
+        <v>57.16</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>6257</v>
@@ -1358,13 +1358,13 @@
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>17.8</v>
+        <v>16.46</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>3.47</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>39.2</v>
+        <v>33.81</v>
       </c>
       <c r="G22" s="1" t="n">
         <v>70</v>
@@ -1458,13 +1458,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>39.49</v>
+        <v>38.69</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>30.88</v>
+        <v>28.6</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>52.35</v>
+        <v>51.57</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>2293</v>
@@ -1490,13 +1490,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>41.52</v>
+        <v>40.47</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>33.08</v>
+        <v>30.6</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>57.1</v>
+        <v>58.75</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>4823</v>
@@ -1522,13 +1522,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>23.63</v>
+        <v>23.9</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0.55</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>44.68</v>
+        <v>44.61</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>868</v>
@@ -1554,20 +1554,20 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>39.44</v>
+        <v>40.57</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>32.8</v>
+        <v>34.08</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>50.25</v>
+        <v>51.53</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>466</v>
       </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>متوسط</t>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1586,13 +1586,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>25.73</v>
+        <v>24.17</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>50.74</v>
+        <v>46.19</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>2048</v>
@@ -1618,13 +1618,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>31.92</v>
+        <v>30.22</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>6.54</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>39.35</v>
+        <v>37.7</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>173</v>
@@ -1650,20 +1650,20 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>38.55</v>
+        <v>41.35</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>29.39</v>
+        <v>31.75</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>55.73</v>
+        <v>60.92</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>7042</v>
       </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>متوسط</t>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1682,13 +1682,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>21.63</v>
+        <v>21.3</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>9.050000000000001</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>42.89</v>
+        <v>41.93</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>66</v>
@@ -1714,20 +1714,20 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>39.59</v>
+        <v>41.06</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>30.19</v>
+        <v>30.15</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>53.27</v>
+        <v>58.02</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>6931</v>
       </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>متوسط</t>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1746,13 +1746,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>42.3</v>
+        <v>41.13</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>31.22</v>
+        <v>31.5</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>56.08</v>
+        <v>55.01</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>5654</v>
@@ -1778,13 +1778,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>36.38</v>
+        <v>36.28</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>3.99</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>54.38</v>
+        <v>52.74</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>16529</v>
@@ -1810,13 +1810,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>34.87</v>
+        <v>35.26</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>4.03</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>51.46</v>
+        <v>50.55</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>5265</v>
@@ -1842,13 +1842,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>41.15</v>
+        <v>41.34</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>32.43</v>
+        <v>32.6</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>54.17</v>
+        <v>55.09</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>2311</v>
@@ -1874,13 +1874,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>42.8</v>
+        <v>42.09</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>34.55</v>
+        <v>33.67</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>55.97</v>
+        <v>55.32</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>1185</v>
@@ -1954,7 +1954,7 @@
         <v>20</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>39049</v>
+        <v>39048</v>
       </c>
       <c r="E2" s="1" t="n">
         <v>4.32</v>
@@ -1973,10 +1973,10 @@
         <v>40</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>531588</v>
+        <v>526146</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>58.76</v>
+        <v>58.15</v>
       </c>
     </row>
     <row r="4">
@@ -1992,10 +1992,10 @@
         <v>60</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>334088</v>
+        <v>339325</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>36.93</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="5">
@@ -2011,10 +2011,10 @@
         <v>80</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>28</v>
+        <v>234</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>0</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Update FIRIS forecast 2026-09-07
</commit_message>
<xml_diff>
--- a/data/report/firis_report.xlsx
+++ b/data/report/firis_report.xlsx
@@ -45,13 +45,13 @@
     <font>
       <name val="B Nazanin"/>
       <b val="1"/>
-      <color rgb="00000000"/>
+      <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="B Nazanin"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="00000000"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -64,7 +64,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FDD835"/>
+        <fgColor rgb="00FB8C00"/>
       </patternFill>
     </fill>
     <fill>
@@ -74,7 +74,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FB8C00"/>
+        <fgColor rgb="00FDD835"/>
       </patternFill>
     </fill>
     <fill>
@@ -127,13 +127,13 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -533,7 +533,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
     </row>
@@ -545,7 +545,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>fli_fars_2026-09-06.tif</t>
+          <t>fli_fars_2026-09-07.tif</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>62.4</v>
+        <v>68.93000000000001</v>
       </c>
     </row>
     <row r="9">
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>37.63</v>
+        <v>41.51</v>
       </c>
     </row>
     <row r="10">
@@ -609,7 +609,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>متوسط</t>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -718,13 +718,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>41.27</v>
+        <v>46.42</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>28.31</v>
+        <v>35.63</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>57.97</v>
+        <v>62.85</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>24441</v>
@@ -750,13 +750,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>41.93</v>
+        <v>45.23</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>27.13</v>
+        <v>30.29</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>56.73</v>
+        <v>61.56</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>5703</v>
@@ -782,13 +782,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>25</v>
+        <v>28.26</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0.43</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>44.97</v>
+        <v>52.44</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>751</v>
@@ -814,13 +814,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>41.76</v>
+        <v>43.33</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>34.3</v>
+        <v>36.03</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>53.09</v>
+        <v>57.26</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>10563</v>
@@ -846,20 +846,20 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>37.52</v>
+        <v>42.73</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>29.05</v>
+        <v>33.86</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>46.54</v>
+        <v>51.39</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>1663</v>
       </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>متوسط</t>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -878,13 +878,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>45.53</v>
+        <v>51.86</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>36.7</v>
+        <v>42.21</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>58.27</v>
+        <v>63.4</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>2137</v>
@@ -910,13 +910,13 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>32.41</v>
+        <v>39.06</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>1.01</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>50.05</v>
+        <v>56.81</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>1950</v>
@@ -942,20 +942,20 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>34.08</v>
+        <v>45.32</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>27.41</v>
+        <v>37.13</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>45.43</v>
+        <v>58.46</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>187</v>
       </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>متوسط</t>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -974,13 +974,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>33.21</v>
+        <v>37.83</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>27.09</v>
+        <v>30.42</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>42.24</v>
+        <v>49.13</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>1059</v>
@@ -1006,13 +1006,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>40.71</v>
+        <v>45.04</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>28.41</v>
+        <v>34.25</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>57.27</v>
+        <v>61.41</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>3976</v>
@@ -1038,13 +1038,13 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>43.25</v>
+        <v>43.57</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>32.11</v>
+        <v>32.21</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>59.44</v>
+        <v>59.49</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>5465</v>
@@ -1070,13 +1070,13 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>41.97</v>
+        <v>42.48</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>28.95</v>
+        <v>28.9</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>61.18</v>
+        <v>61.48</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>6849</v>
@@ -1102,13 +1102,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>25.65</v>
+        <v>26.35</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>1.06</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>38.85</v>
+        <v>38.94</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>79</v>
@@ -1134,13 +1134,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>31.26</v>
+        <v>31.32</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>0.45</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>51.73</v>
+        <v>53.42</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>932</v>
@@ -1166,13 +1166,13 @@
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>42.2</v>
+        <v>43.18</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>31.54</v>
+        <v>33.48</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>57.07</v>
+        <v>58.56</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>4808</v>
@@ -1198,13 +1198,13 @@
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>28.17</v>
+        <v>33.02</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>1.32</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>49.24</v>
+        <v>57.05</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>4944</v>
@@ -1230,20 +1230,20 @@
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>34.89</v>
+        <v>40.42</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>0.65</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>54.18</v>
+        <v>57.1</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>5180</v>
       </c>
-      <c r="H18" s="5" t="inlineStr">
-        <is>
-          <t>متوسط</t>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1262,20 +1262,20 @@
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>38.5</v>
+        <v>43.17</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>0.59</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>54.28</v>
+        <v>61.26</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>3925</v>
       </c>
-      <c r="H19" s="5" t="inlineStr">
-        <is>
-          <t>متوسط</t>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1294,13 +1294,13 @@
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>46.44</v>
+        <v>51.1</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>36.2</v>
+        <v>40.29</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>57.72</v>
+        <v>62.61</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>657</v>
@@ -1326,13 +1326,13 @@
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>43.14</v>
+        <v>45.65</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>30.77</v>
+        <v>33.44</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>59.46</v>
+        <v>60.37</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>6257</v>
@@ -1358,20 +1358,20 @@
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>16.64</v>
+        <v>20.33</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>3.47</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>35.14</v>
+        <v>50.38</v>
       </c>
       <c r="G22" s="1" t="n">
         <v>70</v>
       </c>
-      <c r="H22" s="6" t="inlineStr">
-        <is>
-          <t>کم</t>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -1458,13 +1458,13 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>44.83</v>
+        <v>47.48</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>34.17</v>
+        <v>35.98</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>57.22</v>
+        <v>61.02</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>2293</v>
@@ -1490,20 +1490,20 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>38</v>
+        <v>43.38</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>30.18</v>
+        <v>32.17</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>57.3</v>
+        <v>59.42</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>4823</v>
       </c>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>متوسط</t>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1522,13 +1522,13 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>24.23</v>
+        <v>24.74</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0.55</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>46.86</v>
+        <v>50.76</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>868</v>
@@ -1554,13 +1554,13 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>47.51</v>
+        <v>50.07</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>39.25</v>
+        <v>41.32</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>59.08</v>
+        <v>61.69</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>466</v>
@@ -1586,13 +1586,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>25.95</v>
+        <v>30.61</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>50.89</v>
+        <v>58.26</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>2048</v>
@@ -1618,20 +1618,20 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>32.2</v>
+        <v>40.89</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>6.54</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>39.67</v>
+        <v>49.47</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>173</v>
       </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>متوسط</t>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1650,20 +1650,20 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>37.42</v>
+        <v>42.01</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>28.65</v>
+        <v>31.83</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>54.01</v>
+        <v>60.32</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>7042</v>
       </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>متوسط</t>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1682,13 +1682,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>21.87</v>
+        <v>25.41</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>9.050000000000001</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>42.84</v>
+        <v>52.44</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>66</v>
@@ -1714,13 +1714,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>40.02</v>
+        <v>44.29</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>30.71</v>
+        <v>35.55</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>54.71</v>
+        <v>58.08</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>6931</v>
@@ -1746,13 +1746,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>41.96</v>
+        <v>48.93</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>31.87</v>
+        <v>34.73</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>54.73</v>
+        <v>61.91</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>5654</v>
@@ -1778,20 +1778,20 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>37.59</v>
+        <v>45</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>3.99</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>58.07</v>
+        <v>62.77</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>16529</v>
       </c>
-      <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t>متوسط</t>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1810,20 +1810,20 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>37.35</v>
+        <v>44.42</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>4.03</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>52.81</v>
+        <v>62.55</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>5265</v>
       </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>متوسط</t>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1842,13 +1842,13 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>45.13</v>
+        <v>48.24</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>36.89</v>
+        <v>39.67</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>56.52</v>
+        <v>60.46</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>2311</v>
@@ -1874,13 +1874,13 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>47.28</v>
+        <v>52.96</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>39.34</v>
+        <v>44.3</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>61.23</v>
+        <v>66.38</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>1185</v>
@@ -1973,10 +1973,10 @@
         <v>40</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>497375</v>
+        <v>255646</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>54.97</v>
+        <v>28.26</v>
       </c>
     </row>
     <row r="4">
@@ -1992,10 +1992,10 @@
         <v>60</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>368310</v>
+        <v>608371</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>40.71</v>
+        <v>67.23999999999999</v>
       </c>
     </row>
     <row r="5">
@@ -2011,10 +2011,10 @@
         <v>80</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>20</v>
+        <v>1688</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>0</v>
+        <v>0.19</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Update FIRIS forecast 2026-09-08
</commit_message>
<xml_diff>
--- a/data/report/firis_report.xlsx
+++ b/data/report/firis_report.xlsx
@@ -45,13 +45,13 @@
     <font>
       <name val="B Nazanin"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="00000000"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="B Nazanin"/>
       <b val="1"/>
-      <color rgb="00000000"/>
+      <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -64,7 +64,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FB8C00"/>
+        <fgColor rgb="00FDD835"/>
       </patternFill>
     </fill>
     <fill>
@@ -74,7 +74,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FDD835"/>
+        <fgColor rgb="00FB8C00"/>
       </patternFill>
     </fill>
     <fill>
@@ -127,7 +127,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -533,7 +533,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
     </row>
@@ -545,7 +545,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>fli_fars_2026-09-07.tif</t>
+          <t>fli_fars_2026-09-08.tif</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>68.93000000000001</v>
+        <v>70.19</v>
       </c>
     </row>
     <row r="9">
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>41.51</v>
+        <v>38.18</v>
       </c>
     </row>
     <row r="10">
@@ -609,7 +609,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>زیاد</t>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -718,20 +718,20 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>46.42</v>
+        <v>39.71</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>35.63</v>
+        <v>26.99</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>62.85</v>
+        <v>56.82</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>24441</v>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>زیاد</t>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -750,18 +750,18 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>45.23</v>
+        <v>43.1</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>30.29</v>
+        <v>29.44</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>61.56</v>
+        <v>60.63</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>5703</v>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -782,18 +782,18 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>28.26</v>
+        <v>27.84</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0.43</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>52.44</v>
+        <v>48.06</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>751</v>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -814,18 +814,18 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>43.33</v>
+        <v>45.07</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>36.03</v>
+        <v>37.01</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>57.26</v>
+        <v>57.97</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>10563</v>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -846,20 +846,20 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>42.73</v>
+        <v>36.53</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>33.86</v>
+        <v>28.73</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>51.39</v>
+        <v>45.62</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>1663</v>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>زیاد</t>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -878,18 +878,18 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>51.86</v>
+        <v>46.37</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>42.21</v>
+        <v>37.36</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>63.4</v>
+        <v>57.46</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>2137</v>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -910,20 +910,20 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>39.06</v>
+        <v>40.97</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>1.01</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>56.81</v>
+        <v>60.52</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>1950</v>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>متوسط</t>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -942,20 +942,20 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>45.32</v>
+        <v>34.05</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>37.13</v>
+        <v>27.97</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>58.46</v>
+        <v>45.98</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>187</v>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>زیاد</t>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -974,18 +974,18 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>37.83</v>
+        <v>34.01</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>30.42</v>
+        <v>26.49</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>49.13</v>
+        <v>45.39</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>1059</v>
       </c>
-      <c r="H10" s="5" t="inlineStr">
+      <c r="H10" s="4" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -1006,20 +1006,20 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>45.04</v>
+        <v>39.38</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>34.25</v>
+        <v>28.4</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>61.41</v>
+        <v>55.8</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>3976</v>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>زیاد</t>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -1038,18 +1038,18 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>43.57</v>
+        <v>41.94</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>32.21</v>
+        <v>30.26</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>59.49</v>
+        <v>57.04</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>5465</v>
       </c>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="H12" s="5" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1070,18 +1070,18 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>42.48</v>
+        <v>45.25</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>28.9</v>
+        <v>31.28</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>61.48</v>
+        <v>61.89</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>6849</v>
       </c>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="H13" s="5" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1102,18 +1102,18 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>26.35</v>
+        <v>25.19</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>1.06</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>38.94</v>
+        <v>36.65</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>79</v>
       </c>
-      <c r="H14" s="5" t="inlineStr">
+      <c r="H14" s="4" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -1134,18 +1134,18 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>31.32</v>
+        <v>29.67</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>0.45</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>53.42</v>
+        <v>49.48</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>932</v>
       </c>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="H15" s="4" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -1166,20 +1166,20 @@
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>43.18</v>
+        <v>39.76</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>33.48</v>
+        <v>28.14</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>58.56</v>
+        <v>56.27</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>4808</v>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>زیاد</t>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -1198,7 +1198,7 @@
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>33.02</v>
+        <v>35.13</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>1.32</v>
@@ -1209,7 +1209,7 @@
       <c r="G17" s="1" t="n">
         <v>4944</v>
       </c>
-      <c r="H17" s="5" t="inlineStr">
+      <c r="H17" s="4" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -1230,20 +1230,20 @@
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>40.42</v>
+        <v>33.59</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>0.65</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>57.1</v>
+        <v>49.33</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>5180</v>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>زیاد</t>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -1262,18 +1262,18 @@
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>43.17</v>
+        <v>43.83</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>0.59</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>61.26</v>
+        <v>62.1</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>3925</v>
       </c>
-      <c r="H19" s="4" t="inlineStr">
+      <c r="H19" s="5" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1294,18 +1294,18 @@
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>51.1</v>
+        <v>40.02</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>40.29</v>
+        <v>30.28</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>62.61</v>
+        <v>51.74</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>657</v>
       </c>
-      <c r="H20" s="4" t="inlineStr">
+      <c r="H20" s="5" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1326,18 +1326,18 @@
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>45.65</v>
+        <v>41.64</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>33.44</v>
+        <v>29.56</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>60.37</v>
+        <v>56.43</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>6257</v>
       </c>
-      <c r="H21" s="4" t="inlineStr">
+      <c r="H21" s="5" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1358,20 +1358,20 @@
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>20.33</v>
+        <v>17.56</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>3.47</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>50.38</v>
+        <v>39.23</v>
       </c>
       <c r="G22" s="1" t="n">
         <v>70</v>
       </c>
-      <c r="H22" s="5" t="inlineStr">
-        <is>
-          <t>متوسط</t>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>کم</t>
         </is>
       </c>
     </row>
@@ -1458,20 +1458,20 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>47.48</v>
+        <v>35.1</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>35.98</v>
+        <v>26.33</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>61.02</v>
+        <v>46.81</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>2293</v>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>زیاد</t>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -1490,20 +1490,20 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>43.38</v>
+        <v>38.74</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>32.17</v>
+        <v>29.77</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>59.42</v>
+        <v>56.11</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>4823</v>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>زیاد</t>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -1522,18 +1522,18 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>24.74</v>
+        <v>24.6</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0.55</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>50.76</v>
+        <v>49.97</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>868</v>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -1554,18 +1554,18 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>50.07</v>
+        <v>41.76</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>41.32</v>
+        <v>34.07</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>61.69</v>
+        <v>52.74</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>466</v>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1586,18 +1586,18 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>30.61</v>
+        <v>25.31</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>58.26</v>
+        <v>49.47</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>2048</v>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -1618,20 +1618,20 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>40.89</v>
+        <v>30.4</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>6.54</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>49.47</v>
+        <v>37.63</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>173</v>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>زیاد</t>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -1650,18 +1650,18 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>42.01</v>
+        <v>43.03</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>31.83</v>
+        <v>33.56</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>60.32</v>
+        <v>61.71</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>7042</v>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1682,18 +1682,18 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>25.41</v>
+        <v>23.89</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>9.050000000000001</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>52.44</v>
+        <v>48.06</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>66</v>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -1714,18 +1714,18 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>44.29</v>
+        <v>41.54</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>35.55</v>
+        <v>32</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>58.08</v>
+        <v>56.21</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>6931</v>
       </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1746,20 +1746,20 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>48.93</v>
+        <v>37.34</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>34.73</v>
+        <v>28.42</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>61.91</v>
+        <v>50.35</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>5654</v>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>زیاد</t>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -1778,20 +1778,20 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>45</v>
+        <v>36.56</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>3.99</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>62.77</v>
+        <v>55.21</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>16529</v>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>زیاد</t>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -1810,20 +1810,20 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>44.42</v>
+        <v>36.38</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>4.03</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>62.55</v>
+        <v>52.1</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>5265</v>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>زیاد</t>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -1842,18 +1842,18 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>48.24</v>
+        <v>41.09</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>39.67</v>
+        <v>32.65</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>60.46</v>
+        <v>52.28</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>2311</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H14" s="5" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1874,18 +1874,18 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>52.96</v>
+        <v>43.55</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>44.3</v>
+        <v>35.59</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>66.38</v>
+        <v>57.48</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>1185</v>
       </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="H15" s="5" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1961,7 +1961,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -1973,14 +1973,14 @@
         <v>40</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>255646</v>
+        <v>448088</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>28.26</v>
+        <v>49.53</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1992,10 +1992,10 @@
         <v>60</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>608371</v>
+        <v>415802</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>67.23999999999999</v>
+        <v>45.96</v>
       </c>
     </row>
     <row r="5">
@@ -2011,10 +2011,10 @@
         <v>80</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>1688</v>
+        <v>1815</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>0.19</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Update FIRIS forecast 2026-09-09
</commit_message>
<xml_diff>
--- a/data/report/firis_report.xlsx
+++ b/data/report/firis_report.xlsx
@@ -45,13 +45,13 @@
     <font>
       <name val="B Nazanin"/>
       <b val="1"/>
-      <color rgb="00000000"/>
+      <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="B Nazanin"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="00000000"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -64,7 +64,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FDD835"/>
+        <fgColor rgb="00FB8C00"/>
       </patternFill>
     </fill>
     <fill>
@@ -74,7 +74,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FB8C00"/>
+        <fgColor rgb="00FDD835"/>
       </patternFill>
     </fill>
     <fill>
@@ -127,7 +127,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -533,7 +533,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -545,7 +545,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>fli_fars_2026-09-08.tif</t>
+          <t>fli_fars_2026-09-09.tif</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>70.19</v>
+        <v>68.43000000000001</v>
       </c>
     </row>
     <row r="9">
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>38.18</v>
+        <v>40.44</v>
       </c>
     </row>
     <row r="10">
@@ -609,7 +609,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>متوسط</t>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -718,20 +718,20 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>39.71</v>
+        <v>45.25</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>26.99</v>
+        <v>34.11</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>56.82</v>
+        <v>64.86</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>24441</v>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>متوسط</t>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -750,18 +750,18 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>43.1</v>
+        <v>43.62</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>29.44</v>
+        <v>30.93</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>60.63</v>
+        <v>57.38</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>5703</v>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -782,18 +782,18 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>27.84</v>
+        <v>36.52</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0.43</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>48.06</v>
+        <v>57.32</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>751</v>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -814,18 +814,18 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>45.07</v>
+        <v>41.26</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>37.01</v>
+        <v>33.8</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>57.97</v>
+        <v>54.23</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>10563</v>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -846,18 +846,18 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>36.53</v>
+        <v>39.15</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>28.73</v>
+        <v>31.67</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>45.62</v>
+        <v>48.47</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>1663</v>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -878,18 +878,18 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>46.37</v>
+        <v>53.27</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>37.36</v>
+        <v>43.06</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>57.46</v>
+        <v>66.51000000000001</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>2137</v>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -910,20 +910,20 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>40.97</v>
+        <v>33.65</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>1.01</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>60.52</v>
+        <v>52.71</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>1950</v>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>زیاد</t>
+          <t>متوسط</t>
         </is>
       </c>
     </row>
@@ -942,20 +942,20 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>34.05</v>
+        <v>42.91</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>27.97</v>
+        <v>30.23</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>45.98</v>
+        <v>55.23</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>187</v>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>متوسط</t>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -974,18 +974,18 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>34.01</v>
+        <v>37.89</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>26.49</v>
+        <v>29.12</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>45.39</v>
+        <v>52.66</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>1059</v>
       </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -1006,20 +1006,20 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>39.38</v>
+        <v>41.69</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>28.4</v>
+        <v>28.1</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>55.8</v>
+        <v>59.66</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>3976</v>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>متوسط</t>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1038,18 +1038,18 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>41.94</v>
+        <v>42.45</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>30.26</v>
+        <v>32.14</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>57.04</v>
+        <v>60.02</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>5465</v>
       </c>
-      <c r="H12" s="5" t="inlineStr">
+      <c r="H12" s="4" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1070,18 +1070,18 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>45.25</v>
+        <v>41.65</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>31.28</v>
+        <v>29</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>61.89</v>
+        <v>59.48</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>6849</v>
       </c>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="H13" s="4" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1102,18 +1102,18 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>25.19</v>
+        <v>23.94</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>1.06</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>36.65</v>
+        <v>36.32</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>79</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H14" s="5" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -1134,18 +1134,18 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>29.67</v>
+        <v>29.87</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>0.45</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>49.48</v>
+        <v>51</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>932</v>
       </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="H15" s="5" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -1166,20 +1166,20 @@
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>39.76</v>
+        <v>44.82</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>28.14</v>
+        <v>34.75</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>56.27</v>
+        <v>59.45</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>4808</v>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>متوسط</t>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1198,18 +1198,18 @@
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>35.13</v>
+        <v>31.13</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>1.32</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>57.05</v>
+        <v>52.87</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>4944</v>
       </c>
-      <c r="H17" s="4" t="inlineStr">
+      <c r="H17" s="5" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -1230,20 +1230,20 @@
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>33.59</v>
+        <v>42.74</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>0.65</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>49.33</v>
+        <v>59.21</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>5180</v>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>متوسط</t>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1262,18 +1262,18 @@
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>43.83</v>
+        <v>41.88</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>0.59</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>62.1</v>
+        <v>59.69</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>3925</v>
       </c>
-      <c r="H19" s="5" t="inlineStr">
+      <c r="H19" s="4" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1294,18 +1294,18 @@
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>40.02</v>
+        <v>42.68</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>30.28</v>
+        <v>31.22</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>51.74</v>
+        <v>55.79</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>657</v>
       </c>
-      <c r="H20" s="5" t="inlineStr">
+      <c r="H20" s="4" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1326,18 +1326,18 @@
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>41.64</v>
+        <v>43.63</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>29.56</v>
+        <v>31.3</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>56.43</v>
+        <v>60.69</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>6257</v>
       </c>
-      <c r="H21" s="5" t="inlineStr">
+      <c r="H21" s="4" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1358,13 +1358,13 @@
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>17.56</v>
+        <v>19.93</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>3.47</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>39.23</v>
+        <v>50.53</v>
       </c>
       <c r="G22" s="1" t="n">
         <v>70</v>
@@ -1458,20 +1458,20 @@
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>35.1</v>
+        <v>47.8</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>26.33</v>
+        <v>36.7</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>46.81</v>
+        <v>61.38</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>2293</v>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>متوسط</t>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1490,20 +1490,20 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>38.74</v>
+        <v>44.66</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>29.77</v>
+        <v>35.09</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>56.11</v>
+        <v>61.48</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>4823</v>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>متوسط</t>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1522,18 +1522,18 @@
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>24.6</v>
+        <v>24.95</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>0.55</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>49.97</v>
+        <v>49.88</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>868</v>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -1554,18 +1554,18 @@
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>41.76</v>
+        <v>52.36</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>34.07</v>
+        <v>44.47</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>52.74</v>
+        <v>63.78</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>466</v>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1586,18 +1586,18 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>25.31</v>
+        <v>26.79</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>49.47</v>
+        <v>53.75</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>2048</v>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -1618,18 +1618,18 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>30.4</v>
+        <v>32.6</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>6.54</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>37.63</v>
+        <v>40</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>173</v>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -1650,18 +1650,18 @@
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>43.03</v>
+        <v>40.32</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>33.56</v>
+        <v>29.3</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>61.71</v>
+        <v>58.61</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>7042</v>
       </c>
-      <c r="H8" s="5" t="inlineStr">
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1682,18 +1682,18 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>23.89</v>
+        <v>28.65</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>9.050000000000001</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>48.06</v>
+        <v>57.32</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>66</v>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -1714,18 +1714,18 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>41.54</v>
+        <v>42.79</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>32</v>
+        <v>33.21</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>56.21</v>
+        <v>56.86</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>6931</v>
       </c>
-      <c r="H10" s="5" t="inlineStr">
+      <c r="H10" s="4" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1746,20 +1746,20 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>37.34</v>
+        <v>42.97</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>28.42</v>
+        <v>30.19</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>50.35</v>
+        <v>59.64</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>5654</v>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>متوسط</t>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1778,20 +1778,20 @@
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>36.56</v>
+        <v>41.38</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>3.99</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>55.21</v>
+        <v>61.72</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>16529</v>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>متوسط</t>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1810,20 +1810,20 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>36.38</v>
+        <v>40.63</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>4.03</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>52.1</v>
+        <v>55.82</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>5265</v>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>متوسط</t>
+          <t>زیاد</t>
         </is>
       </c>
     </row>
@@ -1842,18 +1842,18 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>41.09</v>
+        <v>49.07</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>32.65</v>
+        <v>40.79</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>52.28</v>
+        <v>60.42</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>2311</v>
       </c>
-      <c r="H14" s="5" t="inlineStr">
+      <c r="H14" s="4" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1874,18 +1874,18 @@
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>43.55</v>
+        <v>52.09</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>35.59</v>
+        <v>44.64</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>57.48</v>
+        <v>64.65000000000001</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>1185</v>
       </c>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="H15" s="4" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1961,7 +1961,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -1973,14 +1973,14 @@
         <v>40</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>448088</v>
+        <v>328992</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>49.53</v>
+        <v>36.36</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>زیاد</t>
         </is>
@@ -1992,10 +1992,10 @@
         <v>60</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>415802</v>
+        <v>535406</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>45.96</v>
+        <v>59.18</v>
       </c>
     </row>
     <row r="5">
@@ -2011,10 +2011,10 @@
         <v>80</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>1815</v>
+        <v>1307</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>0.2</v>
+        <v>0.14</v>
       </c>
     </row>
     <row r="6">

</xml_diff>